<commit_message>
[BD Log] 2 records — 2026-05-10T23:46
</commit_message>
<xml_diff>
--- a/data/BD_Maintenance_Log.xlsx
+++ b/data/BD_Maintenance_Log.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:L3"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -409,7 +409,8 @@
     <col min="8" max="8" width="35.83203125" customWidth="1"/>
     <col min="9" max="9" width="35.83203125" customWidth="1"/>
     <col min="10" max="10" width="20.83203125" customWidth="1"/>
-    <col min="11" max="11" width="22.83203125" customWidth="1"/>
+    <col min="11" max="11" width="50.83203125" customWidth="1"/>
+    <col min="12" max="12" width="22.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -444,6 +445,9 @@
         <v>사용자재</v>
       </c>
       <c r="K1" t="str">
+        <v>사진URL</v>
+      </c>
+      <c r="L1" t="str">
         <v>등록시간</v>
       </c>
     </row>
@@ -479,12 +483,53 @@
         <v>Roller</v>
       </c>
       <c r="K2" t="str">
+        <v/>
+      </c>
+      <c r="L2" t="str">
         <v>2026-05-08T07:29:25.610Z</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3">
+        <v>1778456764659</v>
+      </c>
+      <c r="B3" t="str">
+        <v>2026-05-10</v>
+      </c>
+      <c r="C3" t="str">
+        <v>CONVEYOR</v>
+      </c>
+      <c r="D3" t="str">
+        <v>08:45</v>
+      </c>
+      <c r="E3" t="str">
+        <v>09:00</v>
+      </c>
+      <c r="F3" t="str">
+        <v>15분</v>
+      </c>
+      <c r="G3">
+        <v>15</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Jam</v>
+      </c>
+      <c r="I3" t="str">
+        <v>Jam</v>
+      </c>
+      <c r="J3" t="str">
+        <v/>
+      </c>
+      <c r="K3" t="str">
+        <v>https://raw.githubusercontent.com/koj260428-sketch/bd-maintenance-log/main/images/1778456764659.jpg</v>
+      </c>
+      <c r="L3" t="str">
+        <v>2026-05-10T23:46:04.659Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
[BD Log] 3 records — 2026-05-11T00:02
</commit_message>
<xml_diff>
--- a/data/BD_Maintenance_Log.xlsx
+++ b/data/BD_Maintenance_Log.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L4"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -527,9 +527,47 @@
         <v>2026-05-10T23:46:04.659Z</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4">
+        <v>1778457742334</v>
+      </c>
+      <c r="B4" t="str">
+        <v>2026-05-11</v>
+      </c>
+      <c r="C4" t="str">
+        <v>CONVEYOR</v>
+      </c>
+      <c r="D4" t="str">
+        <v>09:01</v>
+      </c>
+      <c r="E4" t="str">
+        <v>09:30</v>
+      </c>
+      <c r="F4" t="str">
+        <v>29분</v>
+      </c>
+      <c r="G4">
+        <v>29</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Jam</v>
+      </c>
+      <c r="I4" t="str">
+        <v>Jam</v>
+      </c>
+      <c r="J4" t="str">
+        <v/>
+      </c>
+      <c r="K4" t="str">
+        <v>https://raw.githubusercontent.com/koj260428-sketch/bd-maintenance-log/main/images/1778457742334.jpg</v>
+      </c>
+      <c r="L4" t="str">
+        <v>2026-05-11T00:02:22.334Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
[BD Log] 4 records — 2026-05-11T01:57
</commit_message>
<xml_diff>
--- a/data/BD_Maintenance_Log.xlsx
+++ b/data/BD_Maintenance_Log.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L5"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -565,9 +565,47 @@
         <v>2026-05-11T00:02:22.334Z</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5">
+        <v>1778464654601</v>
+      </c>
+      <c r="B5" t="str">
+        <v>2026-05-11</v>
+      </c>
+      <c r="C5" t="str">
+        <v>CONVEYOR</v>
+      </c>
+      <c r="D5" t="str">
+        <v>10:50</v>
+      </c>
+      <c r="E5" t="str">
+        <v>10:53</v>
+      </c>
+      <c r="F5" t="str">
+        <v>3분</v>
+      </c>
+      <c r="G5">
+        <v>3</v>
+      </c>
+      <c r="H5" t="str">
+        <v>Jam, 테이프가 가이드에 붙음</v>
+      </c>
+      <c r="I5" t="str">
+        <v>카톤 밀어서 Jam 해결, 테이프 제거. Wa02.05.002rf</v>
+      </c>
+      <c r="J5" t="str">
+        <v/>
+      </c>
+      <c r="K5" t="str">
+        <v>https://raw.githubusercontent.com/koj260428-sketch/bd-maintenance-log/main/images/1778464654601.jpg</v>
+      </c>
+      <c r="L5" t="str">
+        <v>2026-05-11T01:57:34.601Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
[BD Log] 5 records — 2026-05-13T04:12
</commit_message>
<xml_diff>
--- a/data/BD_Maintenance_Log.xlsx
+++ b/data/BD_Maintenance_Log.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L6"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -603,9 +603,47 @@
         <v>2026-05-11T01:57:34.601Z</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6">
+        <v>1778645549720</v>
+      </c>
+      <c r="B6" t="str">
+        <v>2026-05-13</v>
+      </c>
+      <c r="C6" t="str">
+        <v>CONVEYOR</v>
+      </c>
+      <c r="D6" t="str">
+        <v>08:00</v>
+      </c>
+      <c r="E6" t="str">
+        <v>11:00</v>
+      </c>
+      <c r="F6" t="str">
+        <v>3시간 0분</v>
+      </c>
+      <c r="G6">
+        <v>180</v>
+      </c>
+      <c r="H6" t="str">
+        <v>Lms에러, 정류기 고장</v>
+      </c>
+      <c r="I6" t="str">
+        <v>모터교체</v>
+      </c>
+      <c r="J6" t="str">
+        <v>모터R57 DRN9OL4/BEZHR/AND8 1.5kw 7.97</v>
+      </c>
+      <c r="K6" t="str">
+        <v/>
+      </c>
+      <c r="L6" t="str">
+        <v>2026-05-13T04:12:29.720Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
[BD Log] 6 records — 2026-05-14T00:09
</commit_message>
<xml_diff>
--- a/data/BD_Maintenance_Log.xlsx
+++ b/data/BD_Maintenance_Log.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L7"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -641,9 +641,47 @@
         <v>2026-05-13T04:12:29.720Z</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7">
+        <v>1778717394680</v>
+      </c>
+      <c r="B7" t="str">
+        <v>2026-05-14</v>
+      </c>
+      <c r="C7" t="str">
+        <v>CONVEYOR</v>
+      </c>
+      <c r="D7" t="str">
+        <v>09:00</v>
+      </c>
+      <c r="E7" t="str">
+        <v>09:05</v>
+      </c>
+      <c r="F7" t="str">
+        <v>5분</v>
+      </c>
+      <c r="G7">
+        <v>5</v>
+      </c>
+      <c r="H7" t="str">
+        <v>Lms에러 1.5.</v>
+      </c>
+      <c r="I7" t="str">
+        <v>Lms 리셋</v>
+      </c>
+      <c r="J7" t="str">
+        <v/>
+      </c>
+      <c r="K7" t="str">
+        <v>https://raw.githubusercontent.com/koj260428-sketch/bd-maintenance-log/main/images/1778717394680.jpg</v>
+      </c>
+      <c r="L7" t="str">
+        <v>2026-05-14T00:09:54.680Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
[BD Log] 3 records — 2026-05-19T03:01
</commit_message>
<xml_diff>
--- a/data/BD_Maintenance_Log.xlsx
+++ b/data/BD_Maintenance_Log.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L4"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -453,235 +453,121 @@
     </row>
     <row r="2">
       <c r="A2">
-        <v>1778225365609</v>
+        <v>1778464654601</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-05-08</v>
+        <v>2026-05-11</v>
       </c>
       <c r="C2" t="str">
         <v>CONVEYOR</v>
       </c>
       <c r="D2" t="str">
-        <v>13:28</v>
+        <v>10:50</v>
       </c>
       <c r="E2" t="str">
-        <v>16:29</v>
+        <v>10:53</v>
       </c>
       <c r="F2" t="str">
-        <v>3시간 1분</v>
+        <v>3분</v>
       </c>
       <c r="G2">
-        <v>181</v>
+        <v>3</v>
       </c>
       <c r="H2" t="str">
-        <v>test 고장</v>
+        <v>Jam, 테이프가 가이드에 붙음</v>
       </c>
       <c r="I2" t="str">
-        <v>test 조치</v>
+        <v>카톤 밀어서 Jam 해결, 테이프 제거. Wa02.05.002rf</v>
       </c>
       <c r="J2" t="str">
-        <v>Roller</v>
+        <v/>
       </c>
       <c r="K2" t="str">
-        <v/>
+        <v>https://raw.githubusercontent.com/koj260428-sketch/bd-maintenance-log/main/images/1778464654601.jpg</v>
       </c>
       <c r="L2" t="str">
-        <v>2026-05-08T07:29:25.610Z</v>
+        <v>2026-05-11T01:57:34.601Z</v>
       </c>
     </row>
     <row r="3">
       <c r="A3">
-        <v>1778456764659</v>
+        <v>1778645549720</v>
       </c>
       <c r="B3" t="str">
-        <v>2026-05-10</v>
+        <v>2026-05-13</v>
       </c>
       <c r="C3" t="str">
         <v>CONVEYOR</v>
       </c>
       <c r="D3" t="str">
-        <v>08:45</v>
+        <v>08:00</v>
       </c>
       <c r="E3" t="str">
-        <v>09:00</v>
+        <v>11:00</v>
       </c>
       <c r="F3" t="str">
-        <v>15분</v>
+        <v>3시간 0분</v>
       </c>
       <c r="G3">
-        <v>15</v>
+        <v>180</v>
       </c>
       <c r="H3" t="str">
-        <v>Jam</v>
+        <v>Lms에러, 정류기 고장</v>
       </c>
       <c r="I3" t="str">
-        <v>Jam</v>
+        <v>모터교체</v>
       </c>
       <c r="J3" t="str">
+        <v>모터R57 DRN9OL4/BEZHR/AND8 1.5kw 7.97</v>
+      </c>
+      <c r="K3" t="str">
         <v/>
       </c>
-      <c r="K3" t="str">
-        <v>https://raw.githubusercontent.com/koj260428-sketch/bd-maintenance-log/main/images/1778456764659.jpg</v>
-      </c>
       <c r="L3" t="str">
-        <v>2026-05-10T23:46:04.659Z</v>
+        <v>2026-05-13T04:12:29.720Z</v>
       </c>
     </row>
     <row r="4">
       <c r="A4">
-        <v>1778457742334</v>
+        <v>1778717394680</v>
       </c>
       <c r="B4" t="str">
-        <v>2026-05-11</v>
+        <v>2026-05-14</v>
       </c>
       <c r="C4" t="str">
         <v>CONVEYOR</v>
       </c>
       <c r="D4" t="str">
-        <v>09:01</v>
+        <v>09:00</v>
       </c>
       <c r="E4" t="str">
-        <v>09:30</v>
+        <v>09:05</v>
       </c>
       <c r="F4" t="str">
-        <v>29분</v>
+        <v>5분</v>
       </c>
       <c r="G4">
-        <v>29</v>
+        <v>5</v>
       </c>
       <c r="H4" t="str">
-        <v>Jam</v>
+        <v>Lms에러 1.5.</v>
       </c>
       <c r="I4" t="str">
-        <v>Jam</v>
+        <v>Lms 리셋</v>
       </c>
       <c r="J4" t="str">
         <v/>
       </c>
       <c r="K4" t="str">
-        <v>https://raw.githubusercontent.com/koj260428-sketch/bd-maintenance-log/main/images/1778457742334.jpg</v>
+        <v>https://raw.githubusercontent.com/koj260428-sketch/bd-maintenance-log/main/images/1778717394680.jpg</v>
       </c>
       <c r="L4" t="str">
-        <v>2026-05-11T00:02:22.334Z</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5">
-        <v>1778464654601</v>
-      </c>
-      <c r="B5" t="str">
-        <v>2026-05-11</v>
-      </c>
-      <c r="C5" t="str">
-        <v>CONVEYOR</v>
-      </c>
-      <c r="D5" t="str">
-        <v>10:50</v>
-      </c>
-      <c r="E5" t="str">
-        <v>10:53</v>
-      </c>
-      <c r="F5" t="str">
-        <v>3분</v>
-      </c>
-      <c r="G5">
-        <v>3</v>
-      </c>
-      <c r="H5" t="str">
-        <v>Jam, 테이프가 가이드에 붙음</v>
-      </c>
-      <c r="I5" t="str">
-        <v>카톤 밀어서 Jam 해결, 테이프 제거. Wa02.05.002rf</v>
-      </c>
-      <c r="J5" t="str">
-        <v/>
-      </c>
-      <c r="K5" t="str">
-        <v>https://raw.githubusercontent.com/koj260428-sketch/bd-maintenance-log/main/images/1778464654601.jpg</v>
-      </c>
-      <c r="L5" t="str">
-        <v>2026-05-11T01:57:34.601Z</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6">
-        <v>1778645549720</v>
-      </c>
-      <c r="B6" t="str">
-        <v>2026-05-13</v>
-      </c>
-      <c r="C6" t="str">
-        <v>CONVEYOR</v>
-      </c>
-      <c r="D6" t="str">
-        <v>08:00</v>
-      </c>
-      <c r="E6" t="str">
-        <v>11:00</v>
-      </c>
-      <c r="F6" t="str">
-        <v>3시간 0분</v>
-      </c>
-      <c r="G6">
-        <v>180</v>
-      </c>
-      <c r="H6" t="str">
-        <v>Lms에러, 정류기 고장</v>
-      </c>
-      <c r="I6" t="str">
-        <v>모터교체</v>
-      </c>
-      <c r="J6" t="str">
-        <v>모터R57 DRN9OL4/BEZHR/AND8 1.5kw 7.97</v>
-      </c>
-      <c r="K6" t="str">
-        <v/>
-      </c>
-      <c r="L6" t="str">
-        <v>2026-05-13T04:12:29.720Z</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7">
-        <v>1778717394680</v>
-      </c>
-      <c r="B7" t="str">
-        <v>2026-05-14</v>
-      </c>
-      <c r="C7" t="str">
-        <v>CONVEYOR</v>
-      </c>
-      <c r="D7" t="str">
-        <v>09:00</v>
-      </c>
-      <c r="E7" t="str">
-        <v>09:05</v>
-      </c>
-      <c r="F7" t="str">
-        <v>5분</v>
-      </c>
-      <c r="G7">
-        <v>5</v>
-      </c>
-      <c r="H7" t="str">
-        <v>Lms에러 1.5.</v>
-      </c>
-      <c r="I7" t="str">
-        <v>Lms 리셋</v>
-      </c>
-      <c r="J7" t="str">
-        <v/>
-      </c>
-      <c r="K7" t="str">
-        <v>https://raw.githubusercontent.com/koj260428-sketch/bd-maintenance-log/main/images/1778717394680.jpg</v>
-      </c>
-      <c r="L7" t="str">
         <v>2026-05-14T00:09:54.680Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
[BD Log] 4 records — 2026-05-19T03:08
</commit_message>
<xml_diff>
--- a/data/BD_Maintenance_Log.xlsx
+++ b/data/BD_Maintenance_Log.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L5"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -565,9 +565,48 @@
         <v>2026-05-14T00:09:54.680Z</v>
       </c>
     </row>
+    <row r="5" xml:space="preserve">
+      <c r="A5">
+        <v>1779160082144</v>
+      </c>
+      <c r="B5" t="str">
+        <v>2026-05-14</v>
+      </c>
+      <c r="C5" t="str">
+        <v>CONVEYOR</v>
+      </c>
+      <c r="D5" t="str">
+        <v>13:30</v>
+      </c>
+      <c r="E5" t="str">
+        <v>15:00</v>
+      </c>
+      <c r="F5" t="str">
+        <v>1시간 30분</v>
+      </c>
+      <c r="G5">
+        <v>90</v>
+      </c>
+      <c r="H5" t="str">
+        <v>롤러 동작 안됨. 롤러 고정볼트 풀림 및 전원선 꼬임으로 파손</v>
+      </c>
+      <c r="I5" t="str" xml:space="preserve">
+        <v xml:space="preserve">롤러교체
+롤러교체 후 Motor module의 error 표시로 Module 교체.</v>
+      </c>
+      <c r="J5" t="str">
+        <v>Motorized roller(10661869_01_0009), Motor module(10662775_01)</v>
+      </c>
+      <c r="K5" t="str">
+        <v/>
+      </c>
+      <c r="L5" t="str">
+        <v>2026-05-19T03:08:02.144Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
[BD Log] 5 records — 2026-06-05T00:20
</commit_message>
<xml_diff>
--- a/data/BD_Maintenance_Log.xlsx
+++ b/data/BD_Maintenance_Log.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L6"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -604,9 +604,47 @@
         <v>2026-05-19T03:08:02.144Z</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6">
+        <v>1780618835158</v>
+      </c>
+      <c r="B6" t="str">
+        <v>2026-06-05</v>
+      </c>
+      <c r="C6" t="str">
+        <v>CONVEYOR</v>
+      </c>
+      <c r="D6" t="str">
+        <v>09:14</v>
+      </c>
+      <c r="E6" t="str">
+        <v>09:17</v>
+      </c>
+      <c r="F6" t="str">
+        <v>3분</v>
+      </c>
+      <c r="G6">
+        <v>3</v>
+      </c>
+      <c r="H6" t="str">
+        <v>센서 틀어짐으로 정지 wa02.05.029ku</v>
+      </c>
+      <c r="I6" t="str">
+        <v>센서 위치 조정</v>
+      </c>
+      <c r="J6" t="str">
+        <v/>
+      </c>
+      <c r="K6" t="str">
+        <v/>
+      </c>
+      <c r="L6" t="str">
+        <v>2026-06-05T00:20:35.158Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
[BD Log] 6 records — 2026-06-05T02:00
</commit_message>
<xml_diff>
--- a/data/BD_Maintenance_Log.xlsx
+++ b/data/BD_Maintenance_Log.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L7"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -642,9 +642,47 @@
         <v>2026-06-05T00:20:35.158Z</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7">
+        <v>1780624801384</v>
+      </c>
+      <c r="B7" t="str">
+        <v>2026-06-05</v>
+      </c>
+      <c r="C7" t="str">
+        <v>CONVEYOR</v>
+      </c>
+      <c r="D7" t="str">
+        <v>10:45</v>
+      </c>
+      <c r="E7" t="str">
+        <v>10:58</v>
+      </c>
+      <c r="F7" t="str">
+        <v>13분</v>
+      </c>
+      <c r="G7">
+        <v>13</v>
+      </c>
+      <c r="H7" t="str">
+        <v>롤러 폴리벨트 풀리 부분 손상 we01.01.008rf</v>
+      </c>
+      <c r="I7" t="str">
+        <v>임시조치; 롤러 2개 연결 끊음</v>
+      </c>
+      <c r="J7" t="str">
+        <v/>
+      </c>
+      <c r="K7" t="str">
+        <v>https://raw.githubusercontent.com/koj260428-sketch/bd-maintenance-log/main/images/1780624801384.jpg</v>
+      </c>
+      <c r="L7" t="str">
+        <v>2026-06-05T02:00:01.384Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
[BD Log] 7 records — 2026-06-08T02:11
</commit_message>
<xml_diff>
--- a/data/BD_Maintenance_Log.xlsx
+++ b/data/BD_Maintenance_Log.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L8"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -680,9 +680,47 @@
         <v>2026-06-05T02:00:01.384Z</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8">
+        <v>1780884665797</v>
+      </c>
+      <c r="B8" t="str">
+        <v>2026-06-08</v>
+      </c>
+      <c r="C8" t="str">
+        <v>CONVEYOR</v>
+      </c>
+      <c r="D8" t="str">
+        <v>11:07</v>
+      </c>
+      <c r="E8" t="str">
+        <v>11:10</v>
+      </c>
+      <c r="F8" t="str">
+        <v>3분</v>
+      </c>
+      <c r="G8">
+        <v>3</v>
+      </c>
+      <c r="H8" t="str">
+        <v>박스 하부 테이프가 가이드레일에 붙어서 걸림</v>
+      </c>
+      <c r="I8" t="str">
+        <v>테이프 정리 및 끼임 해결</v>
+      </c>
+      <c r="J8" t="str">
+        <v/>
+      </c>
+      <c r="K8" t="str">
+        <v>https://raw.githubusercontent.com/koj260428-sketch/bd-maintenance-log/main/images/1780884665797.jpg</v>
+      </c>
+      <c r="L8" t="str">
+        <v>2026-06-08T02:11:05.797Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
[BD Log] 8 records — 2026-06-16T04:23
</commit_message>
<xml_diff>
--- a/data/BD_Maintenance_Log.xlsx
+++ b/data/BD_Maintenance_Log.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L9"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -718,9 +718,47 @@
         <v>2026-06-08T02:11:05.797Z</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9">
+        <v>1781583779973</v>
+      </c>
+      <c r="B9" t="str">
+        <v>2026-06-16</v>
+      </c>
+      <c r="C9" t="str">
+        <v>CONVEYOR</v>
+      </c>
+      <c r="D9" t="str">
+        <v>13:20</v>
+      </c>
+      <c r="E9" t="str">
+        <v>13:25</v>
+      </c>
+      <c r="F9" t="str">
+        <v>5분</v>
+      </c>
+      <c r="G9">
+        <v>5</v>
+      </c>
+      <c r="H9" t="str">
+        <v>카톤 회전 jam</v>
+      </c>
+      <c r="I9" t="str">
+        <v>Jam 카톤 제거</v>
+      </c>
+      <c r="J9" t="str">
+        <v/>
+      </c>
+      <c r="K9" t="str">
+        <v>https://raw.githubusercontent.com/koj260428-sketch/bd-maintenance-log/main/images/1781583779973.jpg</v>
+      </c>
+      <c r="L9" t="str">
+        <v>2026-06-16T04:22:59.973Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L9"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
[BD Log] 9 records — 2026-06-22T00:00
</commit_message>
<xml_diff>
--- a/data/BD_Maintenance_Log.xlsx
+++ b/data/BD_Maintenance_Log.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L10"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -756,9 +756,47 @@
         <v>2026-06-16T04:22:59.973Z</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10">
+        <v>1782086414068</v>
+      </c>
+      <c r="B10" t="str">
+        <v>2026-06-21</v>
+      </c>
+      <c r="C10" t="str">
+        <v>CONVEYOR</v>
+      </c>
+      <c r="D10" t="str">
+        <v>08:55</v>
+      </c>
+      <c r="E10" t="str">
+        <v>08:53</v>
+      </c>
+      <c r="F10" t="str">
+        <v>23시간 58분</v>
+      </c>
+      <c r="G10">
+        <v>1438</v>
+      </c>
+      <c r="H10" t="str">
+        <v>Lms에러</v>
+      </c>
+      <c r="I10" t="str">
+        <v>Lms reset</v>
+      </c>
+      <c r="J10" t="str">
+        <v/>
+      </c>
+      <c r="K10" t="str">
+        <v>https://raw.githubusercontent.com/koj260428-sketch/bd-maintenance-log/main/images/1782086414068.jpg</v>
+      </c>
+      <c r="L10" t="str">
+        <v>2026-06-22T00:00:14.068Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L10"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
[BD Log] 10 records — 2026-07-09T07:01
</commit_message>
<xml_diff>
--- a/data/BD_Maintenance_Log.xlsx
+++ b/data/BD_Maintenance_Log.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L11"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -794,9 +794,47 @@
         <v>2026-06-22T00:00:14.068Z</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11">
+        <v>1783580492593</v>
+      </c>
+      <c r="B11" t="str">
+        <v>2026-07-09</v>
+      </c>
+      <c r="C11" t="str">
+        <v>OTHER</v>
+      </c>
+      <c r="D11" t="str">
+        <v>16:00</v>
+      </c>
+      <c r="E11" t="str">
+        <v>16:00</v>
+      </c>
+      <c r="F11" t="str">
+        <v>0분</v>
+      </c>
+      <c r="G11">
+        <v>0</v>
+      </c>
+      <c r="H11" t="str">
+        <v>화물 1호기 도어 5cm 열린 상태로 소음나면서 정지</v>
+      </c>
+      <c r="I11" t="str">
+        <v>고장접구</v>
+      </c>
+      <c r="J11" t="str">
+        <v/>
+      </c>
+      <c r="K11" t="str">
+        <v>https://raw.githubusercontent.com/koj260428-sketch/bd-maintenance-log/main/images/1783580492593.jpg</v>
+      </c>
+      <c r="L11" t="str">
+        <v>2026-07-09T07:01:32.593Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
[BD Log] 11 records — 2026-07-15T06:19
</commit_message>
<xml_diff>
--- a/data/BD_Maintenance_Log.xlsx
+++ b/data/BD_Maintenance_Log.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L12"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -832,9 +832,47 @@
         <v>2026-07-09T07:01:32.593Z</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12">
+        <v>1784096369403</v>
+      </c>
+      <c r="B12" t="str">
+        <v>2026-07-15</v>
+      </c>
+      <c r="C12" t="str">
+        <v>CONVEYOR</v>
+      </c>
+      <c r="D12" t="str">
+        <v>15:00</v>
+      </c>
+      <c r="E12" t="str">
+        <v>15:10</v>
+      </c>
+      <c r="F12" t="str">
+        <v>10분</v>
+      </c>
+      <c r="G12">
+        <v>10</v>
+      </c>
+      <c r="H12" t="str">
+        <v>We01.01.028rf 롤러 고정브라켓 볼트 풀림으로 롤러 위치 이동 및 선 끼임. 롤러 오류 발생</v>
+      </c>
+      <c r="I12" t="str">
+        <v>롤러 위치 조정 및 브라켓 재고정</v>
+      </c>
+      <c r="J12" t="str">
+        <v/>
+      </c>
+      <c r="K12" t="str">
+        <v/>
+      </c>
+      <c r="L12" t="str">
+        <v>2026-07-15T06:19:29.404Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L12"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
[BD Log] 12 records — 2026-07-16T06:14
</commit_message>
<xml_diff>
--- a/data/BD_Maintenance_Log.xlsx
+++ b/data/BD_Maintenance_Log.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L13"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -870,9 +870,48 @@
         <v>2026-07-15T06:19:29.404Z</v>
       </c>
     </row>
+    <row r="13" xml:space="preserve">
+      <c r="A13">
+        <v>1784182442160</v>
+      </c>
+      <c r="B13" t="str">
+        <v>2026-07-16</v>
+      </c>
+      <c r="C13" t="str">
+        <v>CONVEYOR</v>
+      </c>
+      <c r="D13" t="str">
+        <v>15:10</v>
+      </c>
+      <c r="E13" t="str">
+        <v>15:13</v>
+      </c>
+      <c r="F13" t="str">
+        <v>3분</v>
+      </c>
+      <c r="G13">
+        <v>3</v>
+      </c>
+      <c r="H13" t="str" xml:space="preserve">
+        <v xml:space="preserve">Wa02.01.001sf 방화셔터 구간 카톤 걸림
+카톤이 방화셔터 후단 롤러에 올라탄 상태로 밑면이 닿지않음</v>
+      </c>
+      <c r="I13" t="str">
+        <v>카톤 밀어서 해제</v>
+      </c>
+      <c r="J13" t="str">
+        <v/>
+      </c>
+      <c r="K13" t="str">
+        <v>https://raw.githubusercontent.com/koj260428-sketch/bd-maintenance-log/main/images/1784182442160.jpg</v>
+      </c>
+      <c r="L13" t="str">
+        <v>2026-07-16T06:14:02.161Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L13"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
[BD Log] 13 records — 2026-07-20T07:34
</commit_message>
<xml_diff>
--- a/data/BD_Maintenance_Log.xlsx
+++ b/data/BD_Maintenance_Log.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L14"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -909,9 +909,47 @@
         <v>2026-07-16T06:14:02.161Z</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14">
+        <v>1784532859091</v>
+      </c>
+      <c r="B14" t="str">
+        <v>2026-07-20</v>
+      </c>
+      <c r="C14" t="str">
+        <v>OTHER</v>
+      </c>
+      <c r="D14" t="str">
+        <v>16:28</v>
+      </c>
+      <c r="E14" t="str">
+        <v>16:33</v>
+      </c>
+      <c r="F14" t="str">
+        <v>5분</v>
+      </c>
+      <c r="G14">
+        <v>5</v>
+      </c>
+      <c r="H14" t="str">
+        <v>무게 잉크젯 프린터  와치독 에러로 정지</v>
+      </c>
+      <c r="I14" t="str">
+        <v>헤드 청소 후 재가동</v>
+      </c>
+      <c r="J14" t="str">
+        <v/>
+      </c>
+      <c r="K14" t="str">
+        <v/>
+      </c>
+      <c r="L14" t="str">
+        <v>2026-07-20T07:34:19.091Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L14"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
[BD Log] 14 records — 2026-07-23T04:39
</commit_message>
<xml_diff>
--- a/data/BD_Maintenance_Log.xlsx
+++ b/data/BD_Maintenance_Log.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L15"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -947,9 +947,47 @@
         <v>2026-07-20T07:34:19.091Z</v>
       </c>
     </row>
+    <row r="15">
+      <c r="A15">
+        <v>1784781591640</v>
+      </c>
+      <c r="B15" t="str">
+        <v>2026-07-23</v>
+      </c>
+      <c r="C15" t="str">
+        <v>CONVEYOR</v>
+      </c>
+      <c r="D15" t="str">
+        <v>13:00</v>
+      </c>
+      <c r="E15" t="str">
+        <v>13:35</v>
+      </c>
+      <c r="F15" t="str">
+        <v>35분</v>
+      </c>
+      <c r="G15">
+        <v>35</v>
+      </c>
+      <c r="H15" t="str">
+        <v>Ppi error . 타이밍벨트 끊어짐</v>
+      </c>
+      <c r="I15" t="str">
+        <v>타이밍벨트 교체</v>
+      </c>
+      <c r="J15" t="str">
+        <v>Timing belt 1190 slv14</v>
+      </c>
+      <c r="K15" t="str">
+        <v>https://raw.githubusercontent.com/koj260428-sketch/bd-maintenance-log/main/images/1784781591640.jpg</v>
+      </c>
+      <c r="L15" t="str">
+        <v>2026-07-23T04:39:51.640Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L15"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
[BD Log] 15 records — 2026-07-23T06:06
</commit_message>
<xml_diff>
--- a/data/BD_Maintenance_Log.xlsx
+++ b/data/BD_Maintenance_Log.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L15"/>
+  <dimension ref="A1:L16"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -985,9 +985,47 @@
         <v>2026-07-23T04:39:51.640Z</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16">
+        <v>1784786763252</v>
+      </c>
+      <c r="B16" t="str">
+        <v>2026-07-23</v>
+      </c>
+      <c r="C16" t="str">
+        <v>CONVEYOR</v>
+      </c>
+      <c r="D16" t="str">
+        <v>14:40</v>
+      </c>
+      <c r="E16" t="str">
+        <v>14:55</v>
+      </c>
+      <c r="F16" t="str">
+        <v>15분</v>
+      </c>
+      <c r="G16">
+        <v>15</v>
+      </c>
+      <c r="H16" t="str">
+        <v>밸트 회전 안됨 . 타이밍밸트 파손</v>
+      </c>
+      <c r="I16" t="str">
+        <v>타이밍밸트 교체</v>
+      </c>
+      <c r="J16" t="str">
+        <v>Timing belt sv560</v>
+      </c>
+      <c r="K16" t="str">
+        <v>https://raw.githubusercontent.com/koj260428-sketch/bd-maintenance-log/main/images/1784786763252.jpg</v>
+      </c>
+      <c r="L16" t="str">
+        <v>2026-07-23T06:06:03.252Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L16"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
[BD Log] 16 records — 2026-07-28T02:05
</commit_message>
<xml_diff>
--- a/data/BD_Maintenance_Log.xlsx
+++ b/data/BD_Maintenance_Log.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:L17"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1023,9 +1023,47 @@
         <v>2026-07-23T06:06:03.252Z</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17">
+        <v>1785204320552</v>
+      </c>
+      <c r="B17" t="str">
+        <v>2026-07-28</v>
+      </c>
+      <c r="C17" t="str">
+        <v>OTHER</v>
+      </c>
+      <c r="D17" t="str">
+        <v>11:00</v>
+      </c>
+      <c r="E17" t="str">
+        <v>11:03</v>
+      </c>
+      <c r="F17" t="str">
+        <v>3분</v>
+      </c>
+      <c r="G17">
+        <v>3</v>
+      </c>
+      <c r="H17" t="str">
+        <v>Hba lpn 프린터 인쇄 불량</v>
+      </c>
+      <c r="I17" t="str">
+        <v>노즐 뚫기 버튼으로 조치</v>
+      </c>
+      <c r="J17" t="str">
+        <v/>
+      </c>
+      <c r="K17" t="str">
+        <v/>
+      </c>
+      <c r="L17" t="str">
+        <v>2026-07-28T02:05:20.552Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L17"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
[BD Log] 17 records — 2026-07-31T04:43
</commit_message>
<xml_diff>
--- a/data/BD_Maintenance_Log.xlsx
+++ b/data/BD_Maintenance_Log.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:L18"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1061,9 +1061,47 @@
         <v>2026-07-28T02:05:20.552Z</v>
       </c>
     </row>
+    <row r="18">
+      <c r="A18">
+        <v>1785472989254</v>
+      </c>
+      <c r="B18" t="str">
+        <v>2026-07-31</v>
+      </c>
+      <c r="C18" t="str">
+        <v>CONVEYOR</v>
+      </c>
+      <c r="D18" t="str">
+        <v>11:00</v>
+      </c>
+      <c r="E18" t="str">
+        <v>13:30</v>
+      </c>
+      <c r="F18" t="str">
+        <v>2시간 30분</v>
+      </c>
+      <c r="G18">
+        <v>150</v>
+      </c>
+      <c r="H18" t="str">
+        <v>모터 회전시 감속기 부분 소음발생</v>
+      </c>
+      <c r="I18" t="str">
+        <v>베어링 고장으로 교체 조치</v>
+      </c>
+      <c r="J18" t="str">
+        <v>베어링 6207zz</v>
+      </c>
+      <c r="K18" t="str">
+        <v>https://raw.githubusercontent.com/koj260428-sketch/bd-maintenance-log/main/images/1785472989254.jpg</v>
+      </c>
+      <c r="L18" t="str">
+        <v>2026-07-31T04:43:09.254Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L18"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>